<commit_message>
Automatiza 89 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO RACK GONDOLA.xlsx
+++ b/planilhas/LISTA DE PROCESSO RACK GONDOLA.xlsx
@@ -64,12 +64,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -348,7 +347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -413,7 +412,7 @@
       <c r="E2" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>000666</t>
         </is>
@@ -442,7 +441,7 @@
       <c r="E3" s="3" t="n">
         <v>149</v>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>000667</t>
         </is>
@@ -470,7 +469,7 @@
       <c r="E4" s="3" t="n">
         <v>75</v>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>000668</t>
         </is>
@@ -498,7 +497,7 @@
       <c r="E5" s="3" t="n">
         <v>75</v>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>000669</t>
         </is>
@@ -526,7 +525,7 @@
       <c r="E6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>000670</t>
         </is>
@@ -554,7 +553,7 @@
       <c r="E7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>000671</t>
         </is>
@@ -582,7 +581,7 @@
       <c r="E8" s="3" t="n">
         <v>119</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>000672</t>
         </is>
@@ -610,7 +609,7 @@
       <c r="E9" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>000673</t>
         </is>
@@ -638,7 +637,7 @@
       <c r="E10" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>000674</t>
         </is>
@@ -666,7 +665,7 @@
       <c r="E11" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>000675</t>
         </is>
@@ -694,7 +693,7 @@
       <c r="E12" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>000676</t>
         </is>
@@ -722,7 +721,7 @@
       <c r="E13" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>000677</t>
         </is>
@@ -750,7 +749,7 @@
       <c r="E14" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>000678</t>
         </is>
@@ -778,7 +777,7 @@
       <c r="E15" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>000679</t>
         </is>
@@ -806,7 +805,7 @@
       <c r="E16" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>000680</t>
         </is>
@@ -834,7 +833,7 @@
       <c r="E17" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>000681</t>
         </is>
@@ -862,7 +861,7 @@
       <c r="E18" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>000682</t>
         </is>
@@ -890,7 +889,7 @@
       <c r="E19" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>000683</t>
         </is>
@@ -918,7 +917,7 @@
       <c r="E20" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>000684</t>
         </is>
@@ -946,7 +945,7 @@
       <c r="E21" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>000685</t>
         </is>
@@ -974,7 +973,7 @@
       <c r="E22" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>000686</t>
         </is>
@@ -1002,7 +1001,7 @@
       <c r="E23" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>000687</t>
         </is>
@@ -1030,7 +1029,7 @@
       <c r="E24" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>000688</t>
         </is>
@@ -1058,7 +1057,7 @@
       <c r="E25" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>000689</t>
         </is>
@@ -1086,7 +1085,7 @@
       <c r="E26" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>000690</t>
         </is>
@@ -1114,7 +1113,7 @@
       <c r="E27" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>000691</t>
         </is>
@@ -1142,7 +1141,7 @@
       <c r="E28" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>000692</t>
         </is>
@@ -1170,7 +1169,7 @@
       <c r="E29" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>000693</t>
         </is>
@@ -1198,7 +1197,7 @@
       <c r="E30" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>000694</t>
         </is>
@@ -1226,7 +1225,7 @@
       <c r="E31" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>000695</t>
         </is>
@@ -1254,7 +1253,7 @@
       <c r="E32" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>000696</t>
         </is>
@@ -1282,7 +1281,7 @@
       <c r="E33" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>000697</t>
         </is>
@@ -1310,7 +1309,7 @@
       <c r="E34" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>000698</t>
         </is>
@@ -1338,7 +1337,7 @@
       <c r="E35" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>000699</t>
         </is>
@@ -1366,7 +1365,7 @@
       <c r="E36" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>000700</t>
         </is>
@@ -1394,7 +1393,7 @@
       <c r="E37" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>000701</t>
         </is>
@@ -1422,7 +1421,7 @@
       <c r="E38" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="F38" s="5" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>000702</t>
         </is>
@@ -1450,7 +1449,7 @@
       <c r="E39" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>000703</t>
         </is>
@@ -1478,7 +1477,7 @@
       <c r="E40" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>000704</t>
         </is>
@@ -1506,7 +1505,7 @@
       <c r="E41" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>000705</t>
         </is>
@@ -1534,7 +1533,7 @@
       <c r="E42" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>000706</t>
         </is>
@@ -1562,7 +1561,7 @@
       <c r="E43" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>000707</t>
         </is>
@@ -1590,7 +1589,7 @@
       <c r="E44" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>000708</t>
         </is>
@@ -1618,7 +1617,7 @@
       <c r="E45" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>000709</t>
         </is>
@@ -1646,7 +1645,7 @@
       <c r="E46" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>000710</t>
         </is>
@@ -1674,7 +1673,7 @@
       <c r="E47" s="3" t="n">
         <v>400</v>
       </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>000711</t>
         </is>
@@ -1702,7 +1701,7 @@
       <c r="E48" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="F48" s="5" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>000712</t>
         </is>
@@ -1730,7 +1729,7 @@
       <c r="E49" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr">
         <is>
           <t>000713</t>
         </is>
@@ -1758,7 +1757,7 @@
       <c r="E50" s="3" t="n">
         <v>300</v>
       </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr">
         <is>
           <t>000714</t>
         </is>
@@ -1786,7 +1785,7 @@
       <c r="E51" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr">
         <is>
           <t>000715</t>
         </is>
@@ -1814,7 +1813,7 @@
       <c r="E52" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F52" s="4" t="inlineStr">
         <is>
           <t>000716</t>
         </is>
@@ -1842,7 +1841,7 @@
       <c r="E53" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>000717</t>
         </is>
@@ -1870,7 +1869,7 @@
       <c r="E54" t="n">
         <v>300</v>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>002066</t>
         </is>
@@ -1898,7 +1897,7 @@
       <c r="E55" t="n">
         <v>100</v>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>002067</t>
         </is>
@@ -1926,9 +1925,37 @@
       <c r="E56" t="n">
         <v>100</v>
       </c>
-      <c r="F56" s="5" t="inlineStr">
+      <c r="F56" s="4" t="inlineStr">
         <is>
           <t>002068</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>RACK GONDOLA</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Testeira</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="n">
+        <v>100</v>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>002097</t>
         </is>
       </c>
     </row>

</xml_diff>